<commit_message>
danh gia P2 T3/2026
</commit_message>
<xml_diff>
--- a/members/P2_Form_BP_Cong_Nghe - Hoang.xlsx
+++ b/members/P2_Form_BP_Cong_Nghe - Hoang.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CONG VIEC\project-management\members\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Backup\project-management\members\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42B0AA9-D360-4548-8428-5639BE0CE4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="645" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="TỔNG QUAN &amp; LƯU Ý" sheetId="1" r:id="rId1"/>
     <sheet name="CẤU TRÚC &amp; TRỌNG SỐ" sheetId="2" r:id="rId2"/>
-    <sheet name="ĐÁNH GIÁ HIỆU SUẤT P2" sheetId="3" r:id="rId3"/>
-    <sheet name="MÔ TẢ - PHỤ LỤC" sheetId="4" r:id="rId4"/>
-    <sheet name="NHÂN SỰ" sheetId="6" r:id="rId5"/>
-    <sheet name="Summary_Ranking" sheetId="5" state="hidden" r:id="rId6"/>
+    <sheet name="ĐÁNH GIÁ HIỆU SUẤT P2 T3-2026" sheetId="7" r:id="rId3"/>
+    <sheet name="ĐÁNH GIÁ HIỆU SUẤT P2" sheetId="3" r:id="rId4"/>
+    <sheet name="MÔ TẢ - PHỤ LỤC" sheetId="4" r:id="rId5"/>
+    <sheet name="NHÂN SỰ" sheetId="6" r:id="rId6"/>
+    <sheet name="Summary_Ranking" sheetId="5" state="hidden" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="182">
   <si>
     <t>CẤU TRÚC &amp; TRỌNG SỐ P2+</t>
   </si>
@@ -591,7 +591,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1076,7 +1076,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1198,37 +1198,103 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1257,75 +1323,13 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1346,12 +1350,57 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="25">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFBBF7D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1379,6 +1428,37 @@
           <bgColor rgb="FFFEE2E2"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFEF9C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEDD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
       <fill>
@@ -1450,9 +1530,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1467,53 +1544,53 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Levels_Backend_1" displayName="Levels_Backend_1" ref="A5:D9">
-  <autoFilter ref="A5:D9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Levels_Backend_1" displayName="Levels_Backend_1" ref="A5:D9">
+  <autoFilter ref="A5:D9"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Nhóm năng lực"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Cấp độ 1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Cấp độ 2"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Cấp độ 3"/>
+    <tableColumn id="1" name="Nhóm năng lực"/>
+    <tableColumn id="2" name="Cấp độ 1"/>
+    <tableColumn id="3" name="Cấp độ 2"/>
+    <tableColumn id="4" name="Cấp độ 3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Levels_Designer_2" displayName="Levels_Designer_2" ref="A12:D16">
-  <autoFilter ref="A12:D16" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Levels_Designer_2" displayName="Levels_Designer_2" ref="A12:D16">
+  <autoFilter ref="A12:D16"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Nhóm năng lực"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Cấp độ 1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Cấp độ 2"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Cấp độ 3"/>
+    <tableColumn id="1" name="Nhóm năng lực"/>
+    <tableColumn id="2" name="Cấp độ 1"/>
+    <tableColumn id="3" name="Cấp độ 2"/>
+    <tableColumn id="4" name="Cấp độ 3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Levels_FrontEnd_3" displayName="Levels_FrontEnd_3" ref="A19:D23">
-  <autoFilter ref="A19:D23" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Levels_FrontEnd_3" displayName="Levels_FrontEnd_3" ref="A19:D23">
+  <autoFilter ref="A19:D23"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Nhóm năng lực"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Cấp độ 1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Cấp độ 2"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Cấp độ 3"/>
+    <tableColumn id="1" name="Nhóm năng lực"/>
+    <tableColumn id="2" name="Cấp độ 1"/>
+    <tableColumn id="3" name="Cấp độ 2"/>
+    <tableColumn id="4" name="Cấp độ 3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Levels_FullStack_4" displayName="Levels_FullStack_4" ref="A26:E30">
-  <autoFilter ref="A26:E30" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Levels_FullStack_4" displayName="Levels_FullStack_4" ref="A26:E30">
+  <autoFilter ref="A26:E30"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Nhóm năng lực"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Cấp độ 1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Cấp độ 2"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Cấp độ 3"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Cấp độ 4" dataDxfId="14"/>
+    <tableColumn id="1" name="Nhóm năng lực"/>
+    <tableColumn id="2" name="Cấp độ 1"/>
+    <tableColumn id="3" name="Cấp độ 2"/>
+    <tableColumn id="4" name="Cấp độ 3"/>
+    <tableColumn id="5" name="Cấp độ 4" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1694,7 +1771,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1702,40 +1779,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="3" spans="1:5" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
     </row>
     <row r="5" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
     </row>
     <row r="6" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="65" t="s">
+      <c r="A6" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1749,7 +1826,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1759,240 +1836,240 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="3" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="90" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="81"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="54"/>
     </row>
     <row r="4" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="70"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="56"/>
     </row>
     <row r="5" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="70"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="56"/>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13"/>
-      <c r="B6" s="74" t="s">
+      <c r="B6" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="47"/>
-      <c r="D6" s="70"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="56"/>
     </row>
     <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="13"/>
-      <c r="B7" s="74" t="s">
+      <c r="B7" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="47"/>
-      <c r="D7" s="70"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="56"/>
     </row>
     <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
-      <c r="B8" s="74" t="s">
+      <c r="B8" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="47"/>
-      <c r="D8" s="70"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="56"/>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14"/>
-      <c r="B9" s="76" t="s">
+      <c r="B9" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="77"/>
-      <c r="D9" s="78"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="60"/>
     </row>
     <row r="11" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="84" t="s">
+      <c r="A11" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="55"/>
-      <c r="C11" s="55"/>
-      <c r="D11" s="81"/>
+      <c r="B11" s="53"/>
+      <c r="C11" s="53"/>
+      <c r="D11" s="54"/>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
-      <c r="B12" s="74" t="s">
+      <c r="B12" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="47"/>
-      <c r="D12" s="70"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="56"/>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14"/>
-      <c r="B13" s="76" t="s">
+      <c r="B13" s="65" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="77"/>
-      <c r="D13" s="78"/>
+      <c r="C13" s="59"/>
+      <c r="D13" s="60"/>
     </row>
     <row r="16" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="90" t="s">
+      <c r="A16" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="55"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="81"/>
+      <c r="B16" s="53"/>
+      <c r="C16" s="53"/>
+      <c r="D16" s="54"/>
     </row>
     <row r="17" spans="1:4" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="71" t="s">
+      <c r="A17" s="70" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="47"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="70"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="56"/>
     </row>
     <row r="18" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="91" t="s">
+      <c r="A18" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="77"/>
-      <c r="C18" s="77"/>
-      <c r="D18" s="78"/>
+      <c r="B18" s="59"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="60"/>
     </row>
     <row r="19" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="79" t="s">
+      <c r="A19" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="47"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="47"/>
+      <c r="B19" s="46"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="46"/>
     </row>
     <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="75" t="s">
+      <c r="A20" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="47"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="75" t="s">
+      <c r="A21" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="47"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="47"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
     </row>
     <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="72" t="s">
+      <c r="A22" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
     </row>
     <row r="24" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="83" t="s">
+      <c r="A24" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="47"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
     </row>
     <row r="25" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="80" t="s">
+      <c r="A25" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="55"/>
-      <c r="C25" s="55"/>
-      <c r="D25" s="81"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="54"/>
     </row>
     <row r="26" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="13"/>
-      <c r="B26" s="89" t="s">
+      <c r="B26" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="47"/>
-      <c r="D26" s="70"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="56"/>
     </row>
     <row r="27" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="13"/>
-      <c r="B27" s="89" t="s">
+      <c r="B27" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="47"/>
-      <c r="D27" s="70"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="56"/>
     </row>
     <row r="28" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14"/>
-      <c r="B28" s="88" t="s">
+      <c r="B28" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="C28" s="77"/>
-      <c r="D28" s="78"/>
+      <c r="C28" s="59"/>
+      <c r="D28" s="60"/>
     </row>
     <row r="30" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="80" t="s">
+      <c r="A30" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="55"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="81"/>
+      <c r="B30" s="53"/>
+      <c r="C30" s="53"/>
+      <c r="D30" s="54"/>
     </row>
     <row r="31" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="14"/>
-      <c r="B31" s="88" t="s">
+      <c r="B31" s="58" t="s">
         <v>24</v>
       </c>
-      <c r="C31" s="77"/>
-      <c r="D31" s="78"/>
+      <c r="C31" s="59"/>
+      <c r="D31" s="60"/>
     </row>
     <row r="33" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="80" t="s">
+      <c r="A33" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="B33" s="55"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="81"/>
+      <c r="B33" s="53"/>
+      <c r="C33" s="53"/>
+      <c r="D33" s="54"/>
     </row>
     <row r="34" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="61" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="47"/>
-      <c r="D34" s="70"/>
+      <c r="C34" s="46"/>
+      <c r="D34" s="56"/>
     </row>
     <row r="35" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="14"/>
-      <c r="B35" s="88" t="s">
+      <c r="B35" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="C35" s="77"/>
-      <c r="D35" s="78"/>
+      <c r="C35" s="59"/>
+      <c r="D35" s="60"/>
     </row>
     <row r="36" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="12"/>
     </row>
     <row r="37" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="82" t="s">
+      <c r="A37" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="B37" s="77"/>
-      <c r="C37" s="77"/>
-      <c r="D37" s="77"/>
-      <c r="E37" s="77"/>
+      <c r="B37" s="59"/>
+      <c r="C37" s="59"/>
+      <c r="D37" s="59"/>
+      <c r="E37" s="59"/>
     </row>
     <row r="38" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="26" t="s">
@@ -2084,10 +2161,10 @@
       <c r="B43" s="37"/>
     </row>
     <row r="44" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="85" t="s">
+      <c r="A44" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="86"/>
+      <c r="B44" s="51"/>
     </row>
     <row r="45" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="25" t="s">
@@ -2239,6 +2316,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="B12:D12"/>
@@ -2255,27 +2346,422 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B28:D28"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="25.109375" style="43" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" style="43" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" style="43" customWidth="1"/>
+    <col min="4" max="4" width="25.44140625" style="43" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="43"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="80" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="75"/>
+    </row>
+    <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>181</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="101">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="36" t="str">
+        <f>IF(VLOOKUP(B3,'NHÂN SỰ'!A:B,2,0)=0,"",VLOOKUP(B3,'NHÂN SỰ'!A:B,2,0))</f>
+        <v>Backend</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="41"/>
+    </row>
+    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="77" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="78"/>
+      <c r="C6" s="78"/>
+      <c r="D6" s="75"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="17">
+        <f>IF(B4="",0,INDEX('CẤU TRÚC &amp; TRỌNG SỐ'!B$39:B$42, MATCH(TRIM(B$4), 'CẤU TRÚC &amp; TRỌNG SỐ'!A$39:A$42, 0)))</f>
+        <v>35</v>
+      </c>
+      <c r="C8" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="17">
+        <f>IF(C8="","", B8*VLOOKUP(TRIM(UPPER(C8)), 'CẤU TRÚC &amp; TRỌNG SỐ'!A$51:B$52, 2, FALSE)/100)</f>
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="17">
+        <f>IF(B4="",0,INDEX('CẤU TRÚC &amp; TRỌNG SỐ'!C$39:C$42, MATCH(TRIM(B$4), 'CẤU TRÚC &amp; TRỌNG SỐ'!A$39:A$42, 0)))</f>
+        <v>25</v>
+      </c>
+      <c r="C9" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="17">
+        <f>IF(C9="","", B9*VLOOKUP(TRIM(UPPER(C9)), 'CẤU TRÚC &amp; TRỌNG SỐ'!A$51:B$52, 2, FALSE)/100)</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="17">
+        <f>IF(B4="",0,INDEX('CẤU TRÚC &amp; TRỌNG SỐ'!D$39:D$42, MATCH(TRIM(B$4), 'CẤU TRÚC &amp; TRỌNG SỐ'!A$39:A$42, 0)))</f>
+        <v>15</v>
+      </c>
+      <c r="C10" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="17">
+        <f>IF(C10="","", B10*VLOOKUP(TRIM(UPPER(C10)), 'CẤU TRÚC &amp; TRỌNG SỐ'!A$51:B$52, 2, FALSE)/100)</f>
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="17">
+        <f>IF(B4="",0,INDEX('CẤU TRÚC &amp; TRỌNG SỐ'!E$39:E$42, MATCH(TRIM(B$4), 'CẤU TRÚC &amp; TRỌNG SỐ'!A$39:A$42, 0)))</f>
+        <v>25</v>
+      </c>
+      <c r="C11" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="17">
+        <f>IF(C11="","", B11*VLOOKUP(TRIM(UPPER(C11)), 'CẤU TRÚC &amp; TRỌNG SỐ'!A$51:B$52, 2, FALSE)/100)</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="B12" s="18">
+        <f>SUM(B8:B11)</f>
+        <v>100</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19">
+        <f>IF(OR(D8="", D9="", D10="", D11=""), "", SUM(D8:D11))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="88" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="89"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="20" t="str">
+        <f>IF(D12="","", IF(SUM(D8:D11)&gt;0.8,"ĐẠT","CHƯA ĐẠT"))</f>
+        <v>ĐẠT</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="77" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="78"/>
+      <c r="C15" s="78"/>
+      <c r="D15" s="75"/>
+    </row>
+    <row r="16" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="76" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="75"/>
+    </row>
+    <row r="17" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="83" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="84"/>
+    </row>
+    <row r="18" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="83" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="84"/>
+    </row>
+    <row r="19" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="83" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="84"/>
+    </row>
+    <row r="20" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="85" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="75"/>
+      <c r="C20" s="74">
+        <f>IF(COUNTA(C17:C19)=0,"",
+ IFERROR(VLOOKUP(C17,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B64
++IFERROR(VLOOKUP(C18,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B65
++IFERROR(VLOOKUP(C19,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B66)</f>
+        <v>1</v>
+      </c>
+      <c r="D20" s="75"/>
+    </row>
+    <row r="21" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="33"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="93" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+    </row>
+    <row r="23" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="82" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="75"/>
+      <c r="C23" s="74">
+        <f>IF(OR(D12="",C20=""),"",D12*'CẤU TRÚC &amp; TRỌNG SỐ'!B60+C20*'CẤU TRÚC &amp; TRỌNG SỐ'!B61)</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="75"/>
+    </row>
+    <row r="24" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="91" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="75"/>
+      <c r="C24" s="92" t="str">
+        <f>IF(C23="","KHÔNG CÓ",
+   IF(ROUND(C23,2)&lt;1,"CHƯA ĐẠT",
+         IF(ROUND(C23,2)=1,"ĐẠT","TỐT")
+   )
+)</f>
+        <v>ĐẠT</v>
+      </c>
+      <c r="D24" s="75"/>
+    </row>
+    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="81"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="53"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="86" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="75"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="87" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="78"/>
+      <c r="D27" s="75"/>
+    </row>
+    <row r="28" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B28" s="79" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="78"/>
+      <c r="D28" s="75"/>
+    </row>
+    <row r="29" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" s="79" t="s">
+        <v>95</v>
+      </c>
+      <c r="C29" s="78"/>
+      <c r="D29" s="75"/>
+    </row>
+    <row r="30" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B30" s="79" t="s">
+        <v>97</v>
+      </c>
+      <c r="C30" s="78"/>
+      <c r="D30" s="75"/>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C8:C11">
+    <cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="5" operator="equal">
+      <formula>2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="equal">
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="8" operator="equal">
+      <formula>5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C24">
+    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="TỐT">
+      <formula>NOT(ISERROR(SEARCH("TỐT",C24)))</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="3" priority="2" operator="beginsWith" text="ĐẠT">
+      <formula>LEFT(C24,LEN("ĐẠT"))="ĐẠT"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="CHƯA">
+      <formula>NOT(ISERROR(SEARCH("CHƯA",C24)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D13">
+    <cfRule type="containsText" dxfId="1" priority="9" operator="containsText" text="CHƯA Đạt">
+      <formula>NOT(ISERROR(SEARCH("CHƯA Đạt",D13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="10" operator="containsText" text="ĐẠT">
+      <formula>NOT(ISERROR(SEARCH("ĐẠT",D13)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" sqref="C8:C11">
+      <formula1>"Chưa Đạt,Đạt"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" sqref="C16"/>
+    <dataValidation type="list" allowBlank="1" sqref="C17:C19">
+      <formula1>"Chưa Đạt,Đạt,Tốt"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>'NHÂN SỰ'!$A$2:$A$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>B3</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2286,12 +2772,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="80" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="44"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="75"/>
     </row>
     <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="35" t="s">
@@ -2319,12 +2805,12 @@
       <c r="D4" s="41"/>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="77" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="49"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="44"/>
+      <c r="B6" s="78"/>
+      <c r="C6" s="78"/>
+      <c r="D6" s="75"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
@@ -2419,11 +2905,11 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="62" t="s">
+      <c r="A13" s="88" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="63"/>
-      <c r="C13" s="64"/>
+      <c r="B13" s="89"/>
+      <c r="C13" s="90"/>
       <c r="D13" s="20" t="str">
         <f>IF(D12="","", IF(SUM(D8:D11)&gt;0.8,"ĐẠT","CHƯA ĐẠT"))</f>
         <v>ĐẠT</v>
@@ -2431,12 +2917,12 @@
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="49"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="44"/>
+      <c r="B15" s="78"/>
+      <c r="C15" s="78"/>
+      <c r="D15" s="75"/>
     </row>
     <row r="16" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
@@ -2445,10 +2931,10 @@
       <c r="B16" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="51" t="s">
+      <c r="C16" s="76" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="44"/>
+      <c r="D16" s="75"/>
     </row>
     <row r="17" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="27" t="s">
@@ -2457,10 +2943,10 @@
       <c r="B17" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="57" t="s">
+      <c r="C17" s="83" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="58"/>
+      <c r="D17" s="84"/>
     </row>
     <row r="18" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="27" t="s">
@@ -2469,10 +2955,10 @@
       <c r="B18" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="57" t="s">
+      <c r="C18" s="83" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="58"/>
+      <c r="D18" s="84"/>
     </row>
     <row r="19" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="27" t="s">
@@ -2481,24 +2967,24 @@
       <c r="B19" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="57" t="s">
+      <c r="C19" s="83" t="s">
         <v>44</v>
       </c>
-      <c r="D19" s="58"/>
+      <c r="D19" s="84"/>
     </row>
     <row r="20" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="59" t="s">
+      <c r="A20" s="85" t="s">
         <v>76</v>
       </c>
-      <c r="B20" s="44"/>
-      <c r="C20" s="50">
+      <c r="B20" s="75"/>
+      <c r="C20" s="74">
         <f>IF(COUNTA(C17:C19)=0,"",
  IFERROR(VLOOKUP(C17,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B64
 +IFERROR(VLOOKUP(C18,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B65
 +IFERROR(VLOOKUP(C19,'CẤU TRÚC &amp; TRỌNG SỐ'!A$55:B$57,2,0),0)*'CẤU TRÚC &amp; TRỌNG SỐ'!B66)</f>
         <v>1.07</v>
       </c>
-      <c r="D20" s="44"/>
+      <c r="D20" s="75"/>
     </row>
     <row r="21" spans="1:4" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="33"/>
@@ -2507,30 +2993,30 @@
       <c r="D21" s="34"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="46" t="s">
+      <c r="A22" s="93" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
     </row>
     <row r="23" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="56" t="s">
+      <c r="A23" s="82" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="44"/>
-      <c r="C23" s="50">
+      <c r="B23" s="75"/>
+      <c r="C23" s="74">
         <f>IF(OR(D12="",C20=""),"",D12*'CẤU TRÚC &amp; TRỌNG SỐ'!B60+C20*'CẤU TRÚC &amp; TRỌNG SỐ'!B61)</f>
         <v>1.0350000000000001</v>
       </c>
-      <c r="D23" s="44"/>
+      <c r="D23" s="75"/>
     </row>
     <row r="24" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="91" t="s">
         <v>89</v>
       </c>
-      <c r="B24" s="44"/>
-      <c r="C24" s="45" t="str">
+      <c r="B24" s="75"/>
+      <c r="C24" s="92" t="str">
         <f>IF(C23="","KHÔNG CÓ",
    IF(ROUND(C23,2)&lt;1,"CHƯA ĐẠT",
          IF(ROUND(C23,2)=1,"ĐẠT","TỐT")
@@ -2538,64 +3024,69 @@
 )</f>
         <v>TỐT</v>
       </c>
-      <c r="D24" s="44"/>
+      <c r="D24" s="75"/>
     </row>
     <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="54"/>
-      <c r="B25" s="55"/>
-      <c r="C25" s="55"/>
-      <c r="D25" s="55"/>
+      <c r="A25" s="81"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="53"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="60" t="s">
+      <c r="A26" s="86" t="s">
         <v>90</v>
       </c>
-      <c r="B26" s="49"/>
-      <c r="C26" s="49"/>
-      <c r="D26" s="44"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="75"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="61" t="s">
+      <c r="B27" s="87" t="s">
         <v>80</v>
       </c>
-      <c r="C27" s="49"/>
-      <c r="D27" s="44"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="75"/>
     </row>
     <row r="28" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="B28" s="48" t="s">
+      <c r="B28" s="79" t="s">
         <v>93</v>
       </c>
-      <c r="C28" s="49"/>
-      <c r="D28" s="44"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="75"/>
     </row>
     <row r="29" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B29" s="48" t="s">
+      <c r="B29" s="79" t="s">
         <v>95</v>
       </c>
-      <c r="C29" s="49"/>
-      <c r="D29" s="44"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="75"/>
     </row>
     <row r="30" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="B30" s="48" t="s">
+      <c r="B30" s="79" t="s">
         <v>97</v>
       </c>
-      <c r="C30" s="49"/>
-      <c r="D30" s="44"/>
+      <c r="C30" s="78"/>
+      <c r="D30" s="75"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="A15:D15"/>
@@ -2612,54 +3103,49 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B28:D28"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:C11">
-    <cfRule type="cellIs" dxfId="13" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="4" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="5" operator="equal">
       <formula>2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="6" operator="equal">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="7" operator="equal">
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="8" operator="equal">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C24">
-    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="TỐT">
+    <cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="TỐT">
       <formula>NOT(ISERROR(SEARCH("TỐT",C24)))</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="7" priority="2" operator="beginsWith" text="ĐẠT">
+    <cfRule type="beginsWith" dxfId="18" priority="2" operator="beginsWith" text="ĐẠT">
       <formula>LEFT(C24,LEN("ĐẠT"))="ĐẠT"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="CHƯA">
+    <cfRule type="containsText" dxfId="17" priority="3" operator="containsText" text="CHƯA">
       <formula>NOT(ISERROR(SEARCH("CHƯA",C24)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D13">
-    <cfRule type="containsText" dxfId="5" priority="10" operator="containsText" text="CHƯA Đạt">
+    <cfRule type="containsText" dxfId="16" priority="10" operator="containsText" text="CHƯA Đạt">
       <formula>NOT(ISERROR(SEARCH("CHƯA Đạt",D13)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="12" operator="containsText" text="ĐẠT">
+    <cfRule type="containsText" dxfId="15" priority="12" operator="containsText" text="ĐẠT">
       <formula>NOT(ISERROR(SEARCH("ĐẠT",D13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="C17:C19" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C17:C19">
       <formula1>"Chưa Đạt,Đạt,Tốt"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" sqref="C16" xr:uid="{00000000-0002-0000-0200-000001000000}"/>
-    <dataValidation type="list" allowBlank="1" sqref="C8:C11" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation allowBlank="1" sqref="C16"/>
+    <dataValidation type="list" allowBlank="1" sqref="C8:C11">
       <formula1>"Chưa Đạt,Đạt"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2668,7 +3154,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000004000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>'NHÂN SỰ'!$A$2:$A$7</xm:f>
           </x14:formula1>
@@ -2680,8 +3166,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr applyStyles="1" summaryBelow="0"/>
   </sheetPr>
@@ -2694,28 +3180,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="92" t="s">
+      <c r="A1" s="94" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="96" t="s">
+      <c r="A2" s="98" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
     </row>
     <row r="4" spans="1:4" ht="22.05" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="93" t="s">
+      <c r="A4" s="95" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
     </row>
     <row r="5" spans="1:4" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -2788,12 +3274,12 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="22.05" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="93" t="s">
+      <c r="A11" s="95" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="46"/>
     </row>
     <row r="12" spans="1:4" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -2866,12 +3352,12 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="22.05" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="93" t="s">
+      <c r="A18" s="95" t="s">
         <v>129</v>
       </c>
-      <c r="B18" s="47"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="47"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="46"/>
     </row>
     <row r="19" spans="1:5" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
@@ -2944,13 +3430,13 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="22.05" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="94" t="s">
+      <c r="A25" s="96" t="s">
         <v>142</v>
       </c>
-      <c r="B25" s="95"/>
-      <c r="C25" s="95"/>
-      <c r="D25" s="95"/>
-      <c r="E25" s="95"/>
+      <c r="B25" s="97"/>
+      <c r="C25" s="97"/>
+      <c r="D25" s="97"/>
+      <c r="E25" s="97"/>
     </row>
     <row r="26" spans="1:5" ht="19.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
@@ -3056,8 +3542,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8D0C41-9673-45B2-9EAD-BA190E719E0D}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3126,7 +3612,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0FC5A9D5-3731-4B61-BA5A-0361007D6BD7}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>'CẤU TRÚC &amp; TRỌNG SỐ'!$A$39:$A$42</xm:f>
           </x14:formula1>
@@ -3138,8 +3624,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3155,28 +3641,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="100" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="97" t="s">
+      <c r="A3" s="99" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
     </row>
     <row r="5" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -4264,18 +4750,18 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:E35">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="lessThan">
       <formula>2.5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="between">
       <formula>2.5</formula>
       <formula>3.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="between">
       <formula>3.3</formula>
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>